<commit_message>
fix: new correct excel template sheet
</commit_message>
<xml_diff>
--- a/backend/src/excel-utils/out_excel_sheet_template.xlsx
+++ b/backend/src/excel-utils/out_excel_sheet_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/n.hutchison/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DDD1EEBE-EA35-45D9-9AF2-DCC5D402B3C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9C6AA67A-7B30-4607-AE9B-21829CD1B272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{4108D922-1C2C-8F45-B11F-7B4A4E310542}"/>
   </bookViews>
@@ -967,6 +967,7 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="42" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="42" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="33" borderId="12" xfId="42" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -982,7 +983,6 @@
     <xf numFmtId="0" fontId="27" fillId="33" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="42" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1363,7 +1363,9 @@
   <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.42578125" style="2" customWidth="1"/>
-    <col min="2" max="6" width="12.42578125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="25.28515625" style="2" customWidth="1"/>
+    <col min="4" max="6" width="12.42578125" style="2" customWidth="1"/>
     <col min="7" max="7" width="3.28515625" style="2" customWidth="1"/>
     <col min="8" max="8" width="3.28515625" style="3" customWidth="1"/>
     <col min="9" max="9" width="16" style="2" bestFit="1" customWidth="1"/>
@@ -1548,22 +1550,22 @@
       <c r="H18" s="17"/>
       <c r="I18" s="17"/>
       <c r="J18" s="17"/>
-      <c r="K18" s="29" t="s">
+      <c r="K18" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="L18" s="30"/>
-      <c r="M18" s="30"/>
-      <c r="N18" s="30"/>
-      <c r="O18" s="30"/>
-      <c r="P18" s="30"/>
-      <c r="Q18" s="30"/>
-      <c r="R18" s="30"/>
-      <c r="S18" s="30"/>
-      <c r="T18" s="30"/>
-      <c r="U18" s="30"/>
-      <c r="V18" s="31"/>
+      <c r="L18" s="31"/>
+      <c r="M18" s="31"/>
+      <c r="N18" s="31"/>
+      <c r="O18" s="31"/>
+      <c r="P18" s="31"/>
+      <c r="Q18" s="31"/>
+      <c r="R18" s="31"/>
+      <c r="S18" s="31"/>
+      <c r="T18" s="31"/>
+      <c r="U18" s="31"/>
+      <c r="V18" s="32"/>
       <c r="W18" s="18"/>
-      <c r="X18" s="32" t="s">
+      <c r="X18" s="33" t="s">
         <v>24</v>
       </c>
       <c r="Y18" s="18"/>
@@ -1632,7 +1634,7 @@
         <v>44</v>
       </c>
       <c r="W19" s="19"/>
-      <c r="X19" s="33"/>
+      <c r="X19" s="34"/>
     </row>
     <row r="20" spans="1:25" ht="15" customHeight="1">
       <c r="A20" s="18"/>
@@ -1663,15 +1665,15 @@
     </row>
     <row r="21" spans="1:25" ht="15" customHeight="1">
       <c r="A21" s="18"/>
-      <c r="B21" s="34"/>
-      <c r="C21" s="34"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="34"/>
-      <c r="F21" s="34"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="34"/>
-      <c r="I21" s="34"/>
-      <c r="J21" s="34"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="29"/>
+      <c r="I21" s="29"/>
+      <c r="J21" s="29"/>
       <c r="K21" s="21"/>
       <c r="L21" s="21"/>
       <c r="M21" s="21"/>
@@ -1716,15 +1718,15 @@
     </row>
     <row r="23" spans="1:25">
       <c r="A23" s="18"/>
-      <c r="B23" s="34"/>
-      <c r="C23" s="34"/>
-      <c r="D23" s="34"/>
-      <c r="E23" s="34"/>
-      <c r="F23" s="34"/>
-      <c r="G23" s="34"/>
-      <c r="H23" s="34"/>
-      <c r="I23" s="34"/>
-      <c r="J23" s="34"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="29"/>
+      <c r="H23" s="29"/>
+      <c r="I23" s="29"/>
+      <c r="J23" s="29"/>
       <c r="K23" s="21"/>
       <c r="L23" s="21"/>
       <c r="M23" s="21"/>
@@ -1877,15 +1879,15 @@
     </row>
     <row r="29" spans="1:25">
       <c r="A29" s="18"/>
-      <c r="B29" s="34"/>
-      <c r="C29" s="34"/>
-      <c r="D29" s="34"/>
-      <c r="E29" s="34"/>
-      <c r="F29" s="34"/>
-      <c r="G29" s="34"/>
-      <c r="H29" s="34"/>
-      <c r="I29" s="34"/>
-      <c r="J29" s="34"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="29"/>
+      <c r="H29" s="29"/>
+      <c r="I29" s="29"/>
+      <c r="J29" s="29"/>
       <c r="K29" s="21"/>
       <c r="L29" s="13"/>
       <c r="M29" s="21"/>
@@ -1930,15 +1932,15 @@
     </row>
     <row r="31" spans="1:25">
       <c r="A31" s="18"/>
-      <c r="B31" s="34"/>
-      <c r="C31" s="34"/>
-      <c r="D31" s="34"/>
-      <c r="E31" s="34"/>
-      <c r="F31" s="34"/>
-      <c r="G31" s="34"/>
-      <c r="H31" s="34"/>
-      <c r="I31" s="34"/>
-      <c r="J31" s="34"/>
+      <c r="B31" s="29"/>
+      <c r="C31" s="29"/>
+      <c r="D31" s="29"/>
+      <c r="E31" s="29"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="29"/>
+      <c r="H31" s="29"/>
+      <c r="I31" s="29"/>
+      <c r="J31" s="29"/>
       <c r="K31" s="21"/>
       <c r="L31" s="21"/>
       <c r="M31" s="21"/>
@@ -2010,15 +2012,15 @@
     </row>
     <row r="34" spans="1:25">
       <c r="A34" s="18"/>
-      <c r="B34" s="34"/>
-      <c r="C34" s="34"/>
-      <c r="D34" s="34"/>
-      <c r="E34" s="34"/>
-      <c r="F34" s="34"/>
-      <c r="G34" s="34"/>
-      <c r="H34" s="34"/>
-      <c r="I34" s="34"/>
-      <c r="J34" s="34"/>
+      <c r="B34" s="29"/>
+      <c r="C34" s="29"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="29"/>
+      <c r="G34" s="29"/>
+      <c r="H34" s="29"/>
+      <c r="I34" s="29"/>
+      <c r="J34" s="29"/>
       <c r="K34" s="13"/>
       <c r="L34" s="13"/>
       <c r="M34" s="21"/>
@@ -2063,15 +2065,15 @@
     </row>
     <row r="36" spans="1:25">
       <c r="A36" s="18"/>
-      <c r="B36" s="34"/>
-      <c r="C36" s="34"/>
-      <c r="D36" s="34"/>
-      <c r="E36" s="34"/>
-      <c r="F36" s="34"/>
-      <c r="G36" s="34"/>
-      <c r="H36" s="34"/>
-      <c r="I36" s="34"/>
-      <c r="J36" s="34"/>
+      <c r="B36" s="29"/>
+      <c r="C36" s="29"/>
+      <c r="D36" s="29"/>
+      <c r="E36" s="29"/>
+      <c r="F36" s="29"/>
+      <c r="G36" s="29"/>
+      <c r="H36" s="29"/>
+      <c r="I36" s="29"/>
+      <c r="J36" s="29"/>
       <c r="K36" s="21"/>
       <c r="L36" s="21"/>
       <c r="M36" s="21"/>
@@ -2224,15 +2226,15 @@
     </row>
     <row r="42" spans="1:25">
       <c r="A42" s="18"/>
-      <c r="B42" s="34"/>
-      <c r="C42" s="34"/>
-      <c r="D42" s="34"/>
-      <c r="E42" s="34"/>
-      <c r="F42" s="34"/>
-      <c r="G42" s="34"/>
-      <c r="H42" s="34"/>
-      <c r="I42" s="34"/>
-      <c r="J42" s="34"/>
+      <c r="B42" s="29"/>
+      <c r="C42" s="29"/>
+      <c r="D42" s="29"/>
+      <c r="E42" s="29"/>
+      <c r="F42" s="29"/>
+      <c r="G42" s="29"/>
+      <c r="H42" s="29"/>
+      <c r="I42" s="29"/>
+      <c r="J42" s="29"/>
       <c r="K42" s="21"/>
       <c r="L42" s="13"/>
       <c r="M42" s="21"/>
@@ -2331,15 +2333,15 @@
     </row>
     <row r="46" spans="1:25">
       <c r="A46" s="18"/>
-      <c r="B46" s="34"/>
-      <c r="C46" s="34"/>
-      <c r="D46" s="34"/>
-      <c r="E46" s="34"/>
-      <c r="F46" s="34"/>
-      <c r="G46" s="34"/>
-      <c r="H46" s="34"/>
-      <c r="I46" s="34"/>
-      <c r="J46" s="34"/>
+      <c r="B46" s="29"/>
+      <c r="C46" s="29"/>
+      <c r="D46" s="29"/>
+      <c r="E46" s="29"/>
+      <c r="F46" s="29"/>
+      <c r="G46" s="29"/>
+      <c r="H46" s="29"/>
+      <c r="I46" s="29"/>
+      <c r="J46" s="29"/>
       <c r="K46" s="21"/>
       <c r="L46" s="21"/>
       <c r="M46" s="21"/>
@@ -2384,15 +2386,15 @@
     </row>
     <row r="48" spans="1:25">
       <c r="A48" s="18"/>
-      <c r="B48" s="34"/>
-      <c r="C48" s="34"/>
-      <c r="D48" s="34"/>
-      <c r="E48" s="34"/>
-      <c r="F48" s="34"/>
-      <c r="G48" s="34"/>
-      <c r="H48" s="34"/>
-      <c r="I48" s="34"/>
-      <c r="J48" s="34"/>
+      <c r="B48" s="29"/>
+      <c r="C48" s="29"/>
+      <c r="D48" s="29"/>
+      <c r="E48" s="29"/>
+      <c r="F48" s="29"/>
+      <c r="G48" s="29"/>
+      <c r="H48" s="29"/>
+      <c r="I48" s="29"/>
+      <c r="J48" s="29"/>
       <c r="K48" s="13"/>
       <c r="L48" s="21"/>
       <c r="M48" s="21"/>
@@ -2437,15 +2439,15 @@
     </row>
     <row r="50" spans="1:25">
       <c r="A50" s="18"/>
-      <c r="B50" s="34"/>
-      <c r="C50" s="34"/>
-      <c r="D50" s="34"/>
-      <c r="E50" s="34"/>
-      <c r="F50" s="34"/>
-      <c r="G50" s="34"/>
-      <c r="H50" s="34"/>
-      <c r="I50" s="34"/>
-      <c r="J50" s="34"/>
+      <c r="B50" s="29"/>
+      <c r="C50" s="29"/>
+      <c r="D50" s="29"/>
+      <c r="E50" s="29"/>
+      <c r="F50" s="29"/>
+      <c r="G50" s="29"/>
+      <c r="H50" s="29"/>
+      <c r="I50" s="29"/>
+      <c r="J50" s="29"/>
       <c r="K50" s="21"/>
       <c r="L50" s="21"/>
       <c r="M50" s="21"/>
@@ -2652,15 +2654,15 @@
     </row>
     <row r="58" spans="1:25">
       <c r="A58" s="18"/>
-      <c r="B58" s="34"/>
-      <c r="C58" s="34"/>
-      <c r="D58" s="34"/>
-      <c r="E58" s="34"/>
-      <c r="F58" s="34"/>
-      <c r="G58" s="34"/>
-      <c r="H58" s="34"/>
-      <c r="I58" s="34"/>
-      <c r="J58" s="34"/>
+      <c r="B58" s="29"/>
+      <c r="C58" s="29"/>
+      <c r="D58" s="29"/>
+      <c r="E58" s="29"/>
+      <c r="F58" s="29"/>
+      <c r="G58" s="29"/>
+      <c r="H58" s="29"/>
+      <c r="I58" s="29"/>
+      <c r="J58" s="29"/>
       <c r="K58" s="13"/>
       <c r="L58" s="21"/>
       <c r="M58" s="21"/>
@@ -2732,15 +2734,15 @@
     </row>
     <row r="61" spans="1:25">
       <c r="A61" s="18"/>
-      <c r="B61" s="34"/>
-      <c r="C61" s="34"/>
-      <c r="D61" s="34"/>
-      <c r="E61" s="34"/>
-      <c r="F61" s="34"/>
-      <c r="G61" s="34"/>
-      <c r="H61" s="34"/>
-      <c r="I61" s="34"/>
-      <c r="J61" s="34"/>
+      <c r="B61" s="29"/>
+      <c r="C61" s="29"/>
+      <c r="D61" s="29"/>
+      <c r="E61" s="29"/>
+      <c r="F61" s="29"/>
+      <c r="G61" s="29"/>
+      <c r="H61" s="29"/>
+      <c r="I61" s="29"/>
+      <c r="J61" s="29"/>
       <c r="K61" s="21"/>
       <c r="L61" s="21"/>
       <c r="M61" s="21"/>
@@ -2812,15 +2814,15 @@
     </row>
     <row r="64" spans="1:25">
       <c r="A64" s="18"/>
-      <c r="B64" s="34"/>
-      <c r="C64" s="34"/>
-      <c r="D64" s="34"/>
-      <c r="E64" s="34"/>
-      <c r="F64" s="34"/>
-      <c r="G64" s="34"/>
-      <c r="H64" s="34"/>
-      <c r="I64" s="34"/>
-      <c r="J64" s="34"/>
+      <c r="B64" s="29"/>
+      <c r="C64" s="29"/>
+      <c r="D64" s="29"/>
+      <c r="E64" s="29"/>
+      <c r="F64" s="29"/>
+      <c r="G64" s="29"/>
+      <c r="H64" s="29"/>
+      <c r="I64" s="29"/>
+      <c r="J64" s="29"/>
       <c r="K64" s="21"/>
       <c r="L64" s="21"/>
       <c r="M64" s="21"/>
@@ -2973,15 +2975,15 @@
     </row>
     <row r="70" spans="1:25">
       <c r="A70" s="18"/>
-      <c r="B70" s="34"/>
-      <c r="C70" s="34"/>
-      <c r="D70" s="34"/>
-      <c r="E70" s="34"/>
-      <c r="F70" s="34"/>
-      <c r="G70" s="34"/>
-      <c r="H70" s="34"/>
-      <c r="I70" s="34"/>
-      <c r="J70" s="34"/>
+      <c r="B70" s="29"/>
+      <c r="C70" s="29"/>
+      <c r="D70" s="29"/>
+      <c r="E70" s="29"/>
+      <c r="F70" s="29"/>
+      <c r="G70" s="29"/>
+      <c r="H70" s="29"/>
+      <c r="I70" s="29"/>
+      <c r="J70" s="29"/>
       <c r="K70" s="21"/>
       <c r="L70" s="21"/>
       <c r="M70" s="21"/>
@@ -3134,15 +3136,15 @@
     </row>
     <row r="76" spans="1:25">
       <c r="A76" s="18"/>
-      <c r="B76" s="34"/>
-      <c r="C76" s="34"/>
-      <c r="D76" s="34"/>
-      <c r="E76" s="34"/>
-      <c r="F76" s="34"/>
-      <c r="G76" s="34"/>
-      <c r="H76" s="34"/>
-      <c r="I76" s="34"/>
-      <c r="J76" s="34"/>
+      <c r="B76" s="29"/>
+      <c r="C76" s="29"/>
+      <c r="D76" s="29"/>
+      <c r="E76" s="29"/>
+      <c r="F76" s="29"/>
+      <c r="G76" s="29"/>
+      <c r="H76" s="29"/>
+      <c r="I76" s="29"/>
+      <c r="J76" s="29"/>
       <c r="K76" s="21"/>
       <c r="L76" s="21"/>
       <c r="M76" s="21"/>
@@ -3187,15 +3189,15 @@
     </row>
     <row r="78" spans="1:25">
       <c r="A78" s="18"/>
-      <c r="B78" s="34"/>
-      <c r="C78" s="34"/>
-      <c r="D78" s="34"/>
-      <c r="E78" s="34"/>
-      <c r="F78" s="34"/>
-      <c r="G78" s="34"/>
-      <c r="H78" s="34"/>
-      <c r="I78" s="34"/>
-      <c r="J78" s="34"/>
+      <c r="B78" s="29"/>
+      <c r="C78" s="29"/>
+      <c r="D78" s="29"/>
+      <c r="E78" s="29"/>
+      <c r="F78" s="29"/>
+      <c r="G78" s="29"/>
+      <c r="H78" s="29"/>
+      <c r="I78" s="29"/>
+      <c r="J78" s="29"/>
       <c r="K78" s="13"/>
       <c r="L78" s="21"/>
       <c r="M78" s="21"/>
@@ -3240,15 +3242,15 @@
     </row>
     <row r="80" spans="1:25">
       <c r="A80" s="18"/>
-      <c r="B80" s="34"/>
-      <c r="C80" s="34"/>
-      <c r="D80" s="34"/>
-      <c r="E80" s="34"/>
-      <c r="F80" s="34"/>
-      <c r="G80" s="34"/>
-      <c r="H80" s="34"/>
-      <c r="I80" s="34"/>
-      <c r="J80" s="34"/>
+      <c r="B80" s="29"/>
+      <c r="C80" s="29"/>
+      <c r="D80" s="29"/>
+      <c r="E80" s="29"/>
+      <c r="F80" s="29"/>
+      <c r="G80" s="29"/>
+      <c r="H80" s="29"/>
+      <c r="I80" s="29"/>
+      <c r="J80" s="29"/>
       <c r="K80" s="21"/>
       <c r="L80" s="21"/>
       <c r="M80" s="21"/>
@@ -3455,15 +3457,15 @@
     </row>
     <row r="88" spans="1:25">
       <c r="A88" s="18"/>
-      <c r="B88" s="34"/>
-      <c r="C88" s="34"/>
-      <c r="D88" s="34"/>
-      <c r="E88" s="34"/>
-      <c r="F88" s="34"/>
-      <c r="G88" s="34"/>
-      <c r="H88" s="34"/>
-      <c r="I88" s="34"/>
-      <c r="J88" s="34"/>
+      <c r="B88" s="29"/>
+      <c r="C88" s="29"/>
+      <c r="D88" s="29"/>
+      <c r="E88" s="29"/>
+      <c r="F88" s="29"/>
+      <c r="G88" s="29"/>
+      <c r="H88" s="29"/>
+      <c r="I88" s="29"/>
+      <c r="J88" s="29"/>
       <c r="K88" s="21"/>
       <c r="L88" s="21"/>
       <c r="M88" s="21"/>
@@ -3589,15 +3591,15 @@
     </row>
     <row r="93" spans="1:25">
       <c r="A93" s="18"/>
-      <c r="B93" s="34"/>
-      <c r="C93" s="34"/>
-      <c r="D93" s="34"/>
-      <c r="E93" s="34"/>
-      <c r="F93" s="34"/>
-      <c r="G93" s="34"/>
-      <c r="H93" s="34"/>
-      <c r="I93" s="34"/>
-      <c r="J93" s="34"/>
+      <c r="B93" s="29"/>
+      <c r="C93" s="29"/>
+      <c r="D93" s="29"/>
+      <c r="E93" s="29"/>
+      <c r="F93" s="29"/>
+      <c r="G93" s="29"/>
+      <c r="H93" s="29"/>
+      <c r="I93" s="29"/>
+      <c r="J93" s="29"/>
       <c r="K93" s="21"/>
       <c r="L93" s="13"/>
       <c r="M93" s="21"/>
@@ -3804,15 +3806,15 @@
     </row>
     <row r="101" spans="1:25">
       <c r="A101" s="18"/>
-      <c r="B101" s="34"/>
-      <c r="C101" s="34"/>
-      <c r="D101" s="34"/>
-      <c r="E101" s="34"/>
-      <c r="F101" s="34"/>
-      <c r="G101" s="34"/>
-      <c r="H101" s="34"/>
-      <c r="I101" s="34"/>
-      <c r="J101" s="34"/>
+      <c r="B101" s="29"/>
+      <c r="C101" s="29"/>
+      <c r="D101" s="29"/>
+      <c r="E101" s="29"/>
+      <c r="F101" s="29"/>
+      <c r="G101" s="29"/>
+      <c r="H101" s="29"/>
+      <c r="I101" s="29"/>
+      <c r="J101" s="29"/>
       <c r="K101" s="13"/>
       <c r="L101" s="13"/>
       <c r="M101" s="13"/>
@@ -3857,15 +3859,15 @@
     </row>
     <row r="103" spans="1:25">
       <c r="A103" s="18"/>
-      <c r="B103" s="34"/>
-      <c r="C103" s="34"/>
-      <c r="D103" s="34"/>
-      <c r="E103" s="34"/>
-      <c r="F103" s="34"/>
-      <c r="G103" s="34"/>
-      <c r="H103" s="34"/>
-      <c r="I103" s="34"/>
-      <c r="J103" s="34"/>
+      <c r="B103" s="29"/>
+      <c r="C103" s="29"/>
+      <c r="D103" s="29"/>
+      <c r="E103" s="29"/>
+      <c r="F103" s="29"/>
+      <c r="G103" s="29"/>
+      <c r="H103" s="29"/>
+      <c r="I103" s="29"/>
+      <c r="J103" s="29"/>
       <c r="K103" s="21"/>
       <c r="L103" s="21"/>
       <c r="M103" s="21"/>
@@ -3910,15 +3912,15 @@
     </row>
     <row r="105" spans="1:25">
       <c r="A105" s="18"/>
-      <c r="B105" s="34"/>
-      <c r="C105" s="34"/>
-      <c r="D105" s="34"/>
-      <c r="E105" s="34"/>
-      <c r="F105" s="34"/>
-      <c r="G105" s="34"/>
-      <c r="H105" s="34"/>
-      <c r="I105" s="34"/>
-      <c r="J105" s="34"/>
+      <c r="B105" s="29"/>
+      <c r="C105" s="29"/>
+      <c r="D105" s="29"/>
+      <c r="E105" s="29"/>
+      <c r="F105" s="29"/>
+      <c r="G105" s="29"/>
+      <c r="H105" s="29"/>
+      <c r="I105" s="29"/>
+      <c r="J105" s="29"/>
       <c r="K105" s="21"/>
       <c r="L105" s="21"/>
       <c r="M105" s="21"/>
@@ -3963,15 +3965,15 @@
     </row>
     <row r="107" spans="1:25">
       <c r="A107" s="18"/>
-      <c r="B107" s="34"/>
-      <c r="C107" s="34"/>
-      <c r="D107" s="34"/>
-      <c r="E107" s="34"/>
-      <c r="F107" s="34"/>
-      <c r="G107" s="34"/>
-      <c r="H107" s="34"/>
-      <c r="I107" s="34"/>
-      <c r="J107" s="34"/>
+      <c r="B107" s="29"/>
+      <c r="C107" s="29"/>
+      <c r="D107" s="29"/>
+      <c r="E107" s="29"/>
+      <c r="F107" s="29"/>
+      <c r="G107" s="29"/>
+      <c r="H107" s="29"/>
+      <c r="I107" s="29"/>
+      <c r="J107" s="29"/>
       <c r="K107" s="21"/>
       <c r="L107" s="21"/>
       <c r="M107" s="21"/>
@@ -4016,15 +4018,15 @@
     </row>
     <row r="109" spans="1:25">
       <c r="A109" s="18"/>
-      <c r="B109" s="34"/>
-      <c r="C109" s="34"/>
-      <c r="D109" s="34"/>
-      <c r="E109" s="34"/>
-      <c r="F109" s="34"/>
-      <c r="G109" s="34"/>
-      <c r="H109" s="34"/>
-      <c r="I109" s="34"/>
-      <c r="J109" s="34"/>
+      <c r="B109" s="29"/>
+      <c r="C109" s="29"/>
+      <c r="D109" s="29"/>
+      <c r="E109" s="29"/>
+      <c r="F109" s="29"/>
+      <c r="G109" s="29"/>
+      <c r="H109" s="29"/>
+      <c r="I109" s="29"/>
+      <c r="J109" s="29"/>
       <c r="K109" s="21"/>
       <c r="L109" s="13"/>
       <c r="M109" s="13"/>
@@ -4123,15 +4125,15 @@
     </row>
     <row r="113" spans="1:25">
       <c r="A113" s="18"/>
-      <c r="B113" s="34"/>
-      <c r="C113" s="34"/>
-      <c r="D113" s="34"/>
-      <c r="E113" s="34"/>
-      <c r="F113" s="34"/>
-      <c r="G113" s="34"/>
-      <c r="H113" s="34"/>
-      <c r="I113" s="34"/>
-      <c r="J113" s="34"/>
+      <c r="B113" s="29"/>
+      <c r="C113" s="29"/>
+      <c r="D113" s="29"/>
+      <c r="E113" s="29"/>
+      <c r="F113" s="29"/>
+      <c r="G113" s="29"/>
+      <c r="H113" s="29"/>
+      <c r="I113" s="29"/>
+      <c r="J113" s="29"/>
       <c r="K113" s="13"/>
       <c r="L113" s="21"/>
       <c r="M113" s="21"/>
@@ -4176,15 +4178,15 @@
     </row>
     <row r="115" spans="1:25">
       <c r="A115" s="18"/>
-      <c r="B115" s="34"/>
-      <c r="C115" s="34"/>
-      <c r="D115" s="34"/>
-      <c r="E115" s="34"/>
-      <c r="F115" s="34"/>
-      <c r="G115" s="34"/>
-      <c r="H115" s="34"/>
-      <c r="I115" s="34"/>
-      <c r="J115" s="34"/>
+      <c r="B115" s="29"/>
+      <c r="C115" s="29"/>
+      <c r="D115" s="29"/>
+      <c r="E115" s="29"/>
+      <c r="F115" s="29"/>
+      <c r="G115" s="29"/>
+      <c r="H115" s="29"/>
+      <c r="I115" s="29"/>
+      <c r="J115" s="29"/>
       <c r="K115" s="13"/>
       <c r="L115" s="13"/>
       <c r="M115" s="21"/>
@@ -4229,15 +4231,15 @@
     </row>
     <row r="117" spans="1:25">
       <c r="A117" s="18"/>
-      <c r="B117" s="34"/>
-      <c r="C117" s="34"/>
-      <c r="D117" s="34"/>
-      <c r="E117" s="34"/>
-      <c r="F117" s="34"/>
-      <c r="G117" s="34"/>
-      <c r="H117" s="34"/>
-      <c r="I117" s="34"/>
-      <c r="J117" s="34"/>
+      <c r="B117" s="29"/>
+      <c r="C117" s="29"/>
+      <c r="D117" s="29"/>
+      <c r="E117" s="29"/>
+      <c r="F117" s="29"/>
+      <c r="G117" s="29"/>
+      <c r="H117" s="29"/>
+      <c r="I117" s="29"/>
+      <c r="J117" s="29"/>
       <c r="K117" s="13"/>
       <c r="L117" s="21"/>
       <c r="M117" s="21"/>
@@ -4309,15 +4311,15 @@
     </row>
     <row r="120" spans="1:25">
       <c r="A120" s="18"/>
-      <c r="B120" s="34"/>
-      <c r="C120" s="34"/>
-      <c r="D120" s="34"/>
-      <c r="E120" s="34"/>
-      <c r="F120" s="34"/>
-      <c r="G120" s="34"/>
-      <c r="H120" s="34"/>
-      <c r="I120" s="34"/>
-      <c r="J120" s="34"/>
+      <c r="B120" s="29"/>
+      <c r="C120" s="29"/>
+      <c r="D120" s="29"/>
+      <c r="E120" s="29"/>
+      <c r="F120" s="29"/>
+      <c r="G120" s="29"/>
+      <c r="H120" s="29"/>
+      <c r="I120" s="29"/>
+      <c r="J120" s="29"/>
       <c r="K120" s="21"/>
       <c r="L120" s="21"/>
       <c r="M120" s="21"/>
@@ -4362,15 +4364,15 @@
     </row>
     <row r="122" spans="1:25">
       <c r="A122" s="18"/>
-      <c r="B122" s="34"/>
-      <c r="C122" s="34"/>
-      <c r="D122" s="34"/>
-      <c r="E122" s="34"/>
-      <c r="F122" s="34"/>
-      <c r="G122" s="34"/>
-      <c r="H122" s="34"/>
-      <c r="I122" s="34"/>
-      <c r="J122" s="34"/>
+      <c r="B122" s="29"/>
+      <c r="C122" s="29"/>
+      <c r="D122" s="29"/>
+      <c r="E122" s="29"/>
+      <c r="F122" s="29"/>
+      <c r="G122" s="29"/>
+      <c r="H122" s="29"/>
+      <c r="I122" s="29"/>
+      <c r="J122" s="29"/>
       <c r="K122" s="21"/>
       <c r="L122" s="21"/>
       <c r="M122" s="21"/>
@@ -4469,15 +4471,15 @@
     </row>
     <row r="126" spans="1:25">
       <c r="A126" s="18"/>
-      <c r="B126" s="34"/>
-      <c r="C126" s="34"/>
-      <c r="D126" s="34"/>
-      <c r="E126" s="34"/>
-      <c r="F126" s="34"/>
-      <c r="G126" s="34"/>
-      <c r="H126" s="34"/>
-      <c r="I126" s="34"/>
-      <c r="J126" s="34"/>
+      <c r="B126" s="29"/>
+      <c r="C126" s="29"/>
+      <c r="D126" s="29"/>
+      <c r="E126" s="29"/>
+      <c r="F126" s="29"/>
+      <c r="G126" s="29"/>
+      <c r="H126" s="29"/>
+      <c r="I126" s="29"/>
+      <c r="J126" s="29"/>
       <c r="K126" s="21"/>
       <c r="L126" s="21"/>
       <c r="M126" s="21"/>
@@ -4522,15 +4524,15 @@
     </row>
     <row r="128" spans="1:25">
       <c r="A128" s="18"/>
-      <c r="B128" s="34"/>
-      <c r="C128" s="34"/>
-      <c r="D128" s="34"/>
-      <c r="E128" s="34"/>
-      <c r="F128" s="34"/>
-      <c r="G128" s="34"/>
-      <c r="H128" s="34"/>
-      <c r="I128" s="34"/>
-      <c r="J128" s="34"/>
+      <c r="B128" s="29"/>
+      <c r="C128" s="29"/>
+      <c r="D128" s="29"/>
+      <c r="E128" s="29"/>
+      <c r="F128" s="29"/>
+      <c r="G128" s="29"/>
+      <c r="H128" s="29"/>
+      <c r="I128" s="29"/>
+      <c r="J128" s="29"/>
       <c r="K128" s="13"/>
       <c r="L128" s="13"/>
       <c r="M128" s="21"/>
@@ -4656,15 +4658,15 @@
     </row>
     <row r="133" spans="1:25">
       <c r="A133" s="18"/>
-      <c r="B133" s="34"/>
-      <c r="C133" s="34"/>
-      <c r="D133" s="34"/>
-      <c r="E133" s="34"/>
-      <c r="F133" s="34"/>
-      <c r="G133" s="34"/>
-      <c r="H133" s="34"/>
-      <c r="I133" s="34"/>
-      <c r="J133" s="34"/>
+      <c r="B133" s="29"/>
+      <c r="C133" s="29"/>
+      <c r="D133" s="29"/>
+      <c r="E133" s="29"/>
+      <c r="F133" s="29"/>
+      <c r="G133" s="29"/>
+      <c r="H133" s="29"/>
+      <c r="I133" s="29"/>
+      <c r="J133" s="29"/>
       <c r="K133" s="13"/>
       <c r="L133" s="13"/>
       <c r="M133" s="13"/>
@@ -4925,15 +4927,15 @@
     </row>
     <row r="143" spans="1:25">
       <c r="A143" s="18"/>
-      <c r="B143" s="34"/>
-      <c r="C143" s="34"/>
-      <c r="D143" s="34"/>
-      <c r="E143" s="34"/>
-      <c r="F143" s="34"/>
-      <c r="G143" s="34"/>
-      <c r="H143" s="34"/>
-      <c r="I143" s="34"/>
-      <c r="J143" s="34"/>
+      <c r="B143" s="29"/>
+      <c r="C143" s="29"/>
+      <c r="D143" s="29"/>
+      <c r="E143" s="29"/>
+      <c r="F143" s="29"/>
+      <c r="G143" s="29"/>
+      <c r="H143" s="29"/>
+      <c r="I143" s="29"/>
+      <c r="J143" s="29"/>
       <c r="K143" s="13"/>
       <c r="L143" s="13"/>
       <c r="M143" s="21"/>
@@ -5032,15 +5034,15 @@
     </row>
     <row r="147" spans="1:25">
       <c r="A147" s="18"/>
-      <c r="B147" s="34"/>
-      <c r="C147" s="34"/>
-      <c r="D147" s="34"/>
-      <c r="E147" s="34"/>
-      <c r="F147" s="34"/>
-      <c r="G147" s="34"/>
-      <c r="H147" s="34"/>
-      <c r="I147" s="34"/>
-      <c r="J147" s="34"/>
+      <c r="B147" s="29"/>
+      <c r="C147" s="29"/>
+      <c r="D147" s="29"/>
+      <c r="E147" s="29"/>
+      <c r="F147" s="29"/>
+      <c r="G147" s="29"/>
+      <c r="H147" s="29"/>
+      <c r="I147" s="29"/>
+      <c r="J147" s="29"/>
       <c r="K147" s="21"/>
       <c r="L147" s="21"/>
       <c r="M147" s="21"/>
@@ -5057,43 +5059,9 @@
       <c r="X147" s="18"/>
     </row>
   </sheetData>
-  <mergeCells count="36">
-    <mergeCell ref="B147:J147"/>
-    <mergeCell ref="B107:J107"/>
-    <mergeCell ref="B109:J109"/>
-    <mergeCell ref="B113:J113"/>
-    <mergeCell ref="B115:J115"/>
-    <mergeCell ref="B117:J117"/>
-    <mergeCell ref="B120:J120"/>
-    <mergeCell ref="B122:J122"/>
-    <mergeCell ref="B126:J126"/>
-    <mergeCell ref="B128:J128"/>
-    <mergeCell ref="B133:J133"/>
-    <mergeCell ref="B143:J143"/>
-    <mergeCell ref="B105:J105"/>
-    <mergeCell ref="B58:J58"/>
-    <mergeCell ref="B61:J61"/>
-    <mergeCell ref="B64:J64"/>
-    <mergeCell ref="B70:J70"/>
-    <mergeCell ref="B76:J76"/>
-    <mergeCell ref="B78:J78"/>
-    <mergeCell ref="B80:J80"/>
-    <mergeCell ref="B88:J88"/>
-    <mergeCell ref="B93:J93"/>
-    <mergeCell ref="B101:J101"/>
-    <mergeCell ref="B103:J103"/>
-    <mergeCell ref="B50:J50"/>
+  <mergeCells count="2">
     <mergeCell ref="K18:V18"/>
     <mergeCell ref="X18:X19"/>
-    <mergeCell ref="B21:J21"/>
-    <mergeCell ref="B23:J23"/>
-    <mergeCell ref="B29:J29"/>
-    <mergeCell ref="B31:J31"/>
-    <mergeCell ref="B34:J34"/>
-    <mergeCell ref="B36:J36"/>
-    <mergeCell ref="B42:J42"/>
-    <mergeCell ref="B46:J46"/>
-    <mergeCell ref="B48:J48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>